<commit_message>
feat(03.2-07): ER_FOOTER patcher cluster + 17 JSONL row updates
Add _ER_FOOTER_PATCHES dict + _apply_er_footer_patches() covering the 17
remaining real hallucinations found after Pass-2 regex fix. Each patch
rewrites 'Reference: CCoP 2.0, <wrong>' footers in expected_response to
'Reference: CCoP 2.0 §<correct>' anchored on the row primary
clause_reference.

Covers: B05-002/013/015/016/019, B06-002/013/018/019,
B07-006/007/008/010/015/017/018/027.

Idempotent (re-run = 0 modifications). Timestamped .bak produced.
Regenerates b05/b06/b07 JSONL from patched Excel, preserving Plan 06
authoritative-source + regenerated-consumer pattern.

Post-apply Pass-2 audit: 0 errors, 90 HUMAN_REVIEW (acceptance contract).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ground-truth/expert-validation/CCoP_V2_Test_Cases_Expert_Review.xlsx
+++ b/ground-truth/expert-validation/CCoP_V2_Test_Cases_Expert_Review.xlsx
@@ -8825,7 +8825,7 @@
           <t>According to CCoP 2.0 Section 5.3.1(c), multi-factor authentication requirements are as follows:
 Required for all remote access (critical) Required for privileged accounts (critical) Required for administrative access (critical).
 The intent of this control is to ensure adequate security measures are in place for identity &amp; access management. Organizations must implement controls proportionate to their risk profile while ensuring the core requirements are met.
-Reference: CCoP 2.0, 5.2.3</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L108" s="4" t="inlineStr">
@@ -9701,7 +9701,7 @@
           <t>According to CCoP 2.0 Section 1.6 (Waiver), legacy system exemptions requirements are as follows:
 No blanket exemptions for legacy (critical) Compensating controls required if not compliant (critical) Must document risk and mitigation plan (important).
 The intent of this control is to ensure adequate security measures are in place for system lifecycle. Organizations must implement controls proportionate to their risk profile while ensuring the core requirements are met.
-Reference: CCoP 2.0, 4.3</t>
+Reference: CCoP 2.0 §1.6</t>
         </is>
       </c>
       <c r="L119" s="4" t="inlineStr">
@@ -9861,7 +9861,7 @@
           <t>According to CCoP 2.0 Section 3.8, supply chain control verification requirements are as follows:
 Verify software authenticity and integrity (critical) Source code escrow for critical vendors (important) Vendor security assessment required (critical).
 The intent of this control is to ensure adequate security measures are in place for supply chain security. Organizations must implement controls proportionate to their risk profile while ensuring the core requirements are met.
-Reference: CCoP 2.0, 9.3.1</t>
+Reference: CCoP 2.0 §3.8</t>
         </is>
       </c>
       <c r="L121" s="4" t="inlineStr">
@@ -9941,7 +9941,7 @@
           <t>According to CCoP 2.0 Section 5.11, mobile device management requirements are as follows:
 MDM/EMM solution required (critical) Containerization for corporate data (critical) Remote wipe capability mandatory (important).
 The intent of this control is to ensure adequate security measures are in place for endpoint security. Organizations must implement controls proportionate to their risk profile while ensuring the core requirements are met.
-Reference: CCoP 2.0, 5.3.4</t>
+Reference: CCoP 2.0 §5.11</t>
         </is>
       </c>
       <c r="L122" s="4" t="inlineStr">
@@ -10185,7 +10185,7 @@
           <t>According to CCoP 2.0 Section 5.3.1(c), mfa not required internally requirements are as follows:
 Isolated networks still require MFA (critical) Network isolation is a control, not a waiver (important) All privileged access requires MFA regardless (critical).
 The intent of this control is to ensure adequate security measures are in place for identity &amp; access management. Organizations must implement controls proportionate to their risk profile while ensuring the core requirements are met.
-Reference: CCoP 2.0, 5.2.3</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L125" s="4" t="inlineStr">
@@ -10827,7 +10827,7 @@
 - Protects against phishing and credential theft (critical)
 - Provides layered authentication defense (important)
 Understanding control intent helps in implementing effective security measures that address the underlying threat rather than merely satisfying checkbox requirements. Organizations should consider both the letter and spirit of each control.
-Reference: CCoP 2.0, 5.2.3</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L133" s="4" t="inlineStr">
@@ -11740,7 +11740,7 @@
 - Excessive access increases breach impact (critical)
 - Enforces least privilege over time (important)
 Understanding control intent helps in implementing effective security measures that address the underlying threat rather than merely satisfying checkbox requirements. Organizations should consider both the letter and spirit of each control.
-Reference: CCoP 2.0, 5.2.5</t>
+Reference: CCoP 2.0 §5.2.1</t>
         </is>
       </c>
       <c r="L144" s="4" t="inlineStr">
@@ -12155,7 +12155,7 @@
 - BCP provides recovery path when prevention fails (critical)
 - Addresses availability impact of incidents (important)
 Understanding control intent helps in implementing effective security measures that address the underlying threat rather than merely satisfying checkbox requirements. Organizations should consider both the letter and spirit of each control.
-Reference: CCoP 2.0, 7.4.1</t>
+Reference: CCoP 2.0 §8.2</t>
         </is>
       </c>
       <c r="L149" s="4" t="inlineStr">
@@ -12238,7 +12238,7 @@
 - Risk assessment identifies highest-priority vulnerabilities (critical)
 - Provides basis for control selection and justification (important)
 Understanding control intent helps in implementing effective security measures that address the underlying threat rather than merely satisfying checkbox requirements. Organizations should consider both the letter and spirit of each control.
-Reference: CCoP 2.0, 4.2.1</t>
+Reference: CCoP 2.0 §3.2</t>
         </is>
       </c>
       <c r="L150" s="4" t="inlineStr">
@@ -12855,7 +12855,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.2.4</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L157" s="4" t="inlineStr">
@@ -12944,7 +12944,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.2.5</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L158" s="4" t="inlineStr">
@@ -13033,7 +13033,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.2.4</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L159" s="4" t="inlineStr">
@@ -13207,7 +13207,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.2.6</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L161" s="4" t="inlineStr">
@@ -13648,7 +13648,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 6.3.4</t>
+Reference: CCoP 2.0 §6.2</t>
         </is>
       </c>
       <c r="L166" s="4" t="inlineStr">
@@ -13826,7 +13826,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.4.2</t>
+Reference: CCoP 2.0 §5.5</t>
         </is>
       </c>
       <c r="L168" s="4" t="inlineStr">
@@ -13911,7 +13911,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.4.4</t>
+Reference: CCoP 2.0 §5.7</t>
         </is>
       </c>
       <c r="L169" s="4" t="inlineStr">
@@ -14700,7 +14700,7 @@
 2. Implement compensating controls if immediate remediation not feasible
 3. Establish ongoing monitoring to prevent recurrence
 **Risk Level:** High
-Reference: CCoP 2.0, 5.2.3</t>
+Reference: CCoP 2.0 §5.3.1</t>
         </is>
       </c>
       <c r="L178" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore(03.2): pad B1/B2/B3 test-ids to B01/B02/B03
Normalizes test_id and benchmark_id across the 3 outlier files so every
benchmark in ground-truth/test-suite uses zero-padded identifiers,
matching the filename convention (b01_*, b02_*, b03_*) already in use.

- 80 test_id values rewritten (B[123]-NNN -> B0[123]-NNN)
- 80 benchmark_id values rewritten (B[123] -> B0[123])
- Excel canonical source (Column A Test ID) padded to match

Runtime-neutral: BenchmarkType.short_name already normalizes either
form to non-padded, so CLI flags like --benchmarks B3 continue to work.
Validator passes with 0 errors post-rename.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ground-truth/expert-validation/CCoP_V2_Test_Cases_Expert_Review.xlsx
+++ b/ground-truth/expert-validation/CCoP_V2_Test_Cases_Expert_Review.xlsx
@@ -615,7 +615,7 @@
     <row r="2" ht="225" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>B1-001</t>
+          <t>B01-001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="3" ht="225" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>B1-002</t>
+          <t>B01-002</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="4" ht="210" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>B1-003</t>
+          <t>B01-003</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -846,7 +846,7 @@
     <row r="5" ht="225" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>B1-004</t>
+          <t>B01-004</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -923,7 +923,7 @@
     <row r="6" ht="240" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>B1-005</t>
+          <t>B01-005</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1000,7 +1000,7 @@
     <row r="7" ht="240" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>B1-006</t>
+          <t>B01-006</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1077,7 +1077,7 @@
     <row r="8" ht="225" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>B1-007</t>
+          <t>B01-007</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1154,7 +1154,7 @@
     <row r="9" ht="225" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>B1-008</t>
+          <t>B01-008</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1231,7 +1231,7 @@
     <row r="10" ht="225" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>B1-009</t>
+          <t>B01-009</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1308,7 +1308,7 @@
     <row r="11" ht="255" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>B1-010</t>
+          <t>B01-010</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1385,7 +1385,7 @@
     <row r="12" ht="240" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>B1-011</t>
+          <t>B01-011</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1462,7 +1462,7 @@
     <row r="13" ht="225" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>B1-012</t>
+          <t>B01-012</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="14" ht="255" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>B1-013</t>
+          <t>B01-013</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
     <row r="15" ht="210" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>B1-014</t>
+          <t>B01-014</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1693,7 +1693,7 @@
     <row r="16" ht="225" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>B1-015</t>
+          <t>B01-015</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1770,7 +1770,7 @@
     <row r="17" ht="225" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>B1-016</t>
+          <t>B01-016</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="18" ht="240" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>B1-017</t>
+          <t>B01-017</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="19" ht="225" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>B1-018</t>
+          <t>B01-018</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -2001,7 +2001,7 @@
     <row r="20" ht="240" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>B1-019</t>
+          <t>B01-019</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2078,7 +2078,7 @@
     <row r="21" ht="180" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>B1-020</t>
+          <t>B01-020</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="22" ht="210" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>B1-021</t>
+          <t>B01-021</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2232,7 +2232,7 @@
     <row r="23" ht="225" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>B1-022</t>
+          <t>B01-022</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -2309,7 +2309,7 @@
     <row r="24" ht="240" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>B1-023</t>
+          <t>B01-023</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="25" ht="240" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>B1-024</t>
+          <t>B01-024</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -2463,7 +2463,7 @@
     <row r="26" ht="255" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>B1-025</t>
+          <t>B01-025</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2540,7 +2540,7 @@
     <row r="27" ht="180" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>B2-001</t>
+          <t>B02-001</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2617,7 +2617,7 @@
     <row r="28" ht="180" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>B2-002</t>
+          <t>B02-002</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2694,7 +2694,7 @@
     <row r="29" ht="165" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>B2-003</t>
+          <t>B02-003</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -2771,7 +2771,7 @@
     <row r="30" ht="195" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>B2-004</t>
+          <t>B02-004</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2848,7 +2848,7 @@
     <row r="31" ht="195" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>B2-005</t>
+          <t>B02-005</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -2925,7 +2925,7 @@
     <row r="32" ht="150" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>B2-006</t>
+          <t>B02-006</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -3002,7 +3002,7 @@
     <row r="33" ht="165" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>B2-007</t>
+          <t>B02-007</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -3079,7 +3079,7 @@
     <row r="34" ht="165" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>B2-008</t>
+          <t>B02-008</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -3156,7 +3156,7 @@
     <row r="35" ht="195" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>B2-009</t>
+          <t>B02-009</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -3233,7 +3233,7 @@
     <row r="36" ht="180" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>B2-010</t>
+          <t>B02-010</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -3310,7 +3310,7 @@
     <row r="37" ht="210" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>B2-011</t>
+          <t>B02-011</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -3387,7 +3387,7 @@
     <row r="38" ht="210" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>B2-012</t>
+          <t>B02-012</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -3464,7 +3464,7 @@
     <row r="39" ht="180" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>B2-013</t>
+          <t>B02-013</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -3541,7 +3541,7 @@
     <row r="40" ht="240" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>B2-014</t>
+          <t>B02-014</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3618,7 +3618,7 @@
     <row r="41" ht="225" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>B2-015</t>
+          <t>B02-015</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -3695,7 +3695,7 @@
     <row r="42" ht="225" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>B2-016</t>
+          <t>B02-016</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3772,7 +3772,7 @@
     <row r="43" ht="180" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>B2-017</t>
+          <t>B02-017</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -3849,7 +3849,7 @@
     <row r="44" ht="195" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>B2-018</t>
+          <t>B02-018</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3926,7 +3926,7 @@
     <row r="45" ht="225" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>B2-019</t>
+          <t>B02-019</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -4003,7 +4003,7 @@
     <row r="46" ht="225" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>B2-020</t>
+          <t>B02-020</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -4080,7 +4080,7 @@
     <row r="47" ht="225" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>B2-021</t>
+          <t>B02-021</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="48" ht="195" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>B2-022</t>
+          <t>B02-022</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -4234,7 +4234,7 @@
     <row r="49" ht="210" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>B2-023</t>
+          <t>B02-023</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -4311,7 +4311,7 @@
     <row r="50" ht="240" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>B2-024</t>
+          <t>B02-024</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -4388,7 +4388,7 @@
     <row r="51" ht="240" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>B2-025</t>
+          <t>B02-025</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -4465,7 +4465,7 @@
     <row r="52" ht="150" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>B3-001</t>
+          <t>B03-001</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -4542,7 +4542,7 @@
     <row r="53" ht="150" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>B3-002</t>
+          <t>B03-002</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -4619,7 +4619,7 @@
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>B3-003</t>
+          <t>B03-003</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -4696,7 +4696,7 @@
     <row r="55" ht="75" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>B3-004</t>
+          <t>B03-004</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -4773,7 +4773,7 @@
     <row r="56" ht="75" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>B3-005</t>
+          <t>B03-005</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -4850,7 +4850,7 @@
     <row r="57" ht="75" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>B3-006</t>
+          <t>B03-006</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -4927,7 +4927,7 @@
     <row r="58" ht="75" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>B3-007</t>
+          <t>B03-007</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -5004,7 +5004,7 @@
     <row r="59" ht="75" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>B3-008</t>
+          <t>B03-008</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -5081,7 +5081,7 @@
     <row r="60" ht="75" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>B3-009</t>
+          <t>B03-009</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -5158,7 +5158,7 @@
     <row r="61" ht="60" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>B3-010</t>
+          <t>B03-010</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -5235,7 +5235,7 @@
     <row r="62" ht="75" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>B3-011</t>
+          <t>B03-011</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -5312,7 +5312,7 @@
     <row r="63" ht="75" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>B3-012</t>
+          <t>B03-012</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -5389,7 +5389,7 @@
     <row r="64" ht="90" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>B3-013</t>
+          <t>B03-013</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -5466,7 +5466,7 @@
     <row r="65" ht="75" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>B3-014</t>
+          <t>B03-014</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -5543,7 +5543,7 @@
     <row r="66" ht="75" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>B3-015</t>
+          <t>B03-015</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -5620,7 +5620,7 @@
     <row r="67" ht="60" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>B3-016</t>
+          <t>B03-016</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -5697,7 +5697,7 @@
     <row r="68" ht="75" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>B3-017</t>
+          <t>B03-017</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -5774,7 +5774,7 @@
     <row r="69" ht="75" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>B3-018</t>
+          <t>B03-018</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -5851,7 +5851,7 @@
     <row r="70" ht="75" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>B3-019</t>
+          <t>B03-019</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -5928,7 +5928,7 @@
     <row r="71" ht="75" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>B3-020</t>
+          <t>B03-020</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -6005,7 +6005,7 @@
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>B3-021</t>
+          <t>B03-021</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -6082,7 +6082,7 @@
     <row r="73" ht="75" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>B3-022</t>
+          <t>B03-022</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -6159,7 +6159,7 @@
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>B3-023</t>
+          <t>B03-023</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -6236,7 +6236,7 @@
     <row r="75" ht="75" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>B3-024</t>
+          <t>B03-024</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -6313,7 +6313,7 @@
     <row r="76" ht="75" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>B3-025</t>
+          <t>B03-025</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -6390,7 +6390,7 @@
     <row r="77" ht="75" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>B3-026</t>
+          <t>B03-026</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="78" ht="60" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>B3-027</t>
+          <t>B03-027</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -6544,7 +6544,7 @@
     <row r="79" ht="60" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>B3-028</t>
+          <t>B03-028</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -6621,7 +6621,7 @@
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>B3-029</t>
+          <t>B03-029</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -6694,7 +6694,7 @@
     <row r="81" ht="75" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>B3-030</t>
+          <t>B03-030</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">

</xml_diff>